<commit_message>
Updated for Multispecies model
</commit_message>
<xml_diff>
--- a/MSM/WGNSSK and HAWG 2025/Raw_data/norway_pout_cleaned_and_dequartered.xlsx
+++ b/MSM/WGNSSK and HAWG 2025/Raw_data/norway_pout_cleaned_and_dequartered.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Age-structured-marine-fish-database\MSM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Age-structured-marine-fish-database\MSM\WGNSSK and HAWG 2025\Raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1104BC-BEFE-4A49-8416-B4D1D5BDDBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2174B4-A8E3-4FCC-A237-6FED6065B490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-16110" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E39FE445-15FF-4EEB-AEB3-75FB5B747230}"/>
+    <workbookView xWindow="28680" yWindow="-16110" windowWidth="29040" windowHeight="15720" xr2:uid="{E39FE445-15FF-4EEB-AEB3-75FB5B747230}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 10.3.3 Num" sheetId="1" r:id="rId1"/>
@@ -54,8 +54,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -135,7 +135,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -144,10 +144,10 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -156,31 +156,31 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="3" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="3" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="3" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" indent="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -519,14 +519,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{902D435B-E7EE-467F-8940-7B1AA4334FAE}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="9.140625" style="19"/>
+    <col min="1" max="5" width="9.140625" style="19"/>
+    <col min="6" max="6" width="10.140625" style="19" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -548,719 +549,845 @@
       <c r="J1" s="19"/>
       <c r="K1" s="19"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="19">
         <v>1984</v>
       </c>
       <c r="B2" s="19">
-        <v>43360</v>
+        <v>43360000</v>
       </c>
       <c r="C2" s="19">
-        <v>23292</v>
+        <v>23292000</v>
       </c>
       <c r="D2" s="19">
-        <v>3709</v>
+        <v>3709000</v>
       </c>
       <c r="E2" s="19">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>275000</v>
+      </c>
+      <c r="F2"/>
+      <c r="L2"/>
+      <c r="M2"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="19">
         <v>1985</v>
       </c>
       <c r="B3" s="19">
-        <v>31869</v>
+        <v>31869000</v>
       </c>
       <c r="C3" s="19">
-        <v>11536</v>
+        <v>11536000</v>
       </c>
       <c r="D3" s="19">
-        <v>1874</v>
+        <v>1874000</v>
       </c>
       <c r="E3" s="19">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>268000</v>
+      </c>
+      <c r="F3"/>
+      <c r="L3"/>
+      <c r="M3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>1986</v>
       </c>
       <c r="B4" s="19">
-        <v>54438</v>
+        <v>54438000</v>
       </c>
       <c r="C4" s="19">
-        <v>8624</v>
+        <v>8624000</v>
       </c>
       <c r="D4" s="19">
-        <v>1184</v>
+        <v>1184000</v>
       </c>
       <c r="E4" s="19">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>148000</v>
+      </c>
+      <c r="F4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="19">
         <v>1987</v>
       </c>
       <c r="B5" s="19">
-        <v>11511</v>
+        <v>11511000</v>
       </c>
       <c r="C5" s="19">
-        <v>17561</v>
+        <v>17561000</v>
       </c>
       <c r="D5" s="19">
-        <v>1079</v>
+        <v>1079000</v>
       </c>
       <c r="E5" s="19">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>135000</v>
+      </c>
+      <c r="F5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>1988</v>
       </c>
       <c r="B6" s="19">
-        <v>52192</v>
+        <v>52192000</v>
       </c>
       <c r="C6" s="19">
-        <v>3624</v>
+        <v>3624000</v>
       </c>
       <c r="D6" s="19">
-        <v>2925</v>
+        <v>2925000</v>
       </c>
       <c r="E6" s="19">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>105000</v>
+      </c>
+      <c r="F6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="19">
         <v>1989</v>
       </c>
       <c r="B7" s="19">
-        <v>53853</v>
+        <v>53853000</v>
       </c>
       <c r="C7" s="19">
-        <v>15524</v>
+        <v>15524000</v>
       </c>
       <c r="D7" s="19">
-        <v>832</v>
+        <v>832000</v>
       </c>
       <c r="E7" s="19">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>453000</v>
+      </c>
+      <c r="F7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>1990</v>
       </c>
       <c r="B8" s="19">
-        <v>65695</v>
+        <v>65695000</v>
       </c>
       <c r="C8" s="19">
-        <v>15593</v>
+        <v>15593000</v>
       </c>
       <c r="D8" s="19">
-        <v>2313</v>
+        <v>2313000</v>
       </c>
       <c r="E8" s="19">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>184000</v>
+      </c>
+      <c r="F8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="19">
         <v>1991</v>
       </c>
       <c r="B9" s="19">
-        <v>118615</v>
+        <v>118615000</v>
       </c>
       <c r="C9" s="19">
-        <v>19692</v>
+        <v>19692000</v>
       </c>
       <c r="D9" s="19">
-        <v>2770</v>
+        <v>2770000</v>
       </c>
       <c r="E9" s="19">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>310000</v>
+      </c>
+      <c r="F9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>1992</v>
       </c>
       <c r="B10" s="19">
-        <v>63393</v>
+        <v>63393000</v>
       </c>
       <c r="C10" s="19">
-        <v>35503</v>
+        <v>35503000</v>
       </c>
       <c r="D10" s="19">
-        <v>4319</v>
+        <v>4319000</v>
       </c>
       <c r="E10" s="19">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>506000</v>
+      </c>
+      <c r="F10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="19">
         <v>1993</v>
       </c>
       <c r="B11" s="19">
-        <v>55142</v>
+        <v>55142000</v>
       </c>
       <c r="C11" s="19">
-        <v>16696</v>
+        <v>16696000</v>
       </c>
       <c r="D11" s="19">
-        <v>5438</v>
+        <v>5438000</v>
       </c>
       <c r="E11" s="19">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>798000</v>
+      </c>
+      <c r="F11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>1994</v>
       </c>
       <c r="B12" s="19">
-        <v>158931</v>
+        <v>158931000</v>
       </c>
       <c r="C12" s="19">
-        <v>14523</v>
+        <v>14523000</v>
       </c>
       <c r="D12" s="19">
-        <v>2567</v>
+        <v>2567000</v>
       </c>
       <c r="E12" s="19">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>646000</v>
+      </c>
+      <c r="F12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="19">
         <v>1995</v>
       </c>
       <c r="B13" s="19">
-        <v>63422</v>
+        <v>63422000</v>
       </c>
       <c r="C13" s="19">
-        <v>49143</v>
+        <v>49143000</v>
       </c>
       <c r="D13" s="19">
-        <v>2912</v>
+        <v>2912000</v>
       </c>
       <c r="E13" s="19">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>612000</v>
+      </c>
+      <c r="F13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>1996</v>
       </c>
       <c r="B14" s="19">
-        <v>132726</v>
+        <v>132726000</v>
       </c>
       <c r="C14" s="19">
-        <v>18044</v>
+        <v>18044000</v>
       </c>
       <c r="D14" s="19">
-        <v>9576</v>
+        <v>9576000</v>
       </c>
       <c r="E14" s="19">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>627000</v>
+      </c>
+      <c r="F14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="19">
         <v>1997</v>
       </c>
       <c r="B15" s="19">
-        <v>27199</v>
+        <v>27199000</v>
       </c>
       <c r="C15" s="19">
-        <v>43331</v>
+        <v>43331000</v>
       </c>
       <c r="D15" s="19">
-        <v>4120</v>
+        <v>4120000</v>
       </c>
       <c r="E15" s="19">
-        <v>1797</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1797000</v>
+      </c>
+      <c r="F15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>1998</v>
       </c>
       <c r="B16" s="19">
-        <v>48968</v>
+        <v>48968000</v>
       </c>
       <c r="C16" s="19">
-        <v>8502</v>
+        <v>8502000</v>
       </c>
       <c r="D16" s="19">
-        <v>9188</v>
+        <v>9188000</v>
       </c>
       <c r="E16" s="19">
-        <v>878</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>878000</v>
+      </c>
+      <c r="F16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19">
         <v>1999</v>
       </c>
       <c r="B17" s="19">
-        <v>114193</v>
+        <v>114193000</v>
       </c>
       <c r="C17" s="19">
-        <v>16904</v>
+        <v>16904000</v>
       </c>
       <c r="D17" s="19">
-        <v>2181</v>
+        <v>2181000</v>
       </c>
       <c r="E17" s="19">
-        <v>1719</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1719000</v>
+      </c>
+      <c r="F17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>2000</v>
       </c>
       <c r="B18" s="19">
-        <v>31461</v>
+        <v>31461000</v>
       </c>
       <c r="C18" s="19">
-        <v>40660</v>
+        <v>40660000</v>
       </c>
       <c r="D18" s="19">
-        <v>4544</v>
+        <v>4544000</v>
       </c>
       <c r="E18" s="19">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>564000</v>
+      </c>
+      <c r="F18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="19">
         <v>2001</v>
       </c>
       <c r="B19" s="19">
-        <v>32532</v>
+        <v>32532000</v>
       </c>
       <c r="C19" s="19">
-        <v>8892</v>
+        <v>8892000</v>
       </c>
       <c r="D19" s="19">
-        <v>7941</v>
+        <v>7941000</v>
       </c>
       <c r="E19" s="19">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>877000</v>
+      </c>
+      <c r="F19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>2002</v>
       </c>
       <c r="B20" s="19">
-        <v>24775</v>
+        <v>24775000</v>
       </c>
       <c r="C20" s="19">
-        <v>10089</v>
+        <v>10089000</v>
       </c>
       <c r="D20" s="19">
-        <v>1892</v>
+        <v>1892000</v>
       </c>
       <c r="E20" s="19">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1500000</v>
+      </c>
+      <c r="F20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="19">
         <v>2003</v>
       </c>
       <c r="B21" s="19">
-        <v>9561</v>
+        <v>9561000</v>
       </c>
       <c r="C21" s="19">
-        <v>6199</v>
+        <v>6199000</v>
       </c>
       <c r="D21" s="19">
-        <v>1856</v>
+        <v>1856000</v>
       </c>
       <c r="E21" s="19">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+        <v>470000</v>
+      </c>
+      <c r="F21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>2004</v>
       </c>
       <c r="B22" s="19">
-        <v>9506</v>
+        <v>9506000</v>
       </c>
       <c r="C22" s="19">
-        <v>2924</v>
+        <v>2924000</v>
       </c>
       <c r="D22" s="19">
-        <v>1387</v>
+        <v>1387000</v>
       </c>
       <c r="E22" s="19">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>334000</v>
+      </c>
+      <c r="F22"/>
+      <c r="L22"/>
+      <c r="M22"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="19">
         <v>2005</v>
       </c>
       <c r="B23" s="19">
-        <v>36824</v>
+        <v>36824000</v>
       </c>
       <c r="C23" s="19">
-        <v>2962</v>
+        <v>2962000</v>
       </c>
       <c r="D23" s="19">
-        <v>717</v>
+        <v>717000</v>
       </c>
       <c r="E23" s="19">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <v>304000</v>
+      </c>
+      <c r="F23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>2006</v>
       </c>
       <c r="B24" s="19">
-        <v>27626</v>
+        <v>27626000</v>
       </c>
       <c r="C24" s="19">
-        <v>11757</v>
+        <v>11757000</v>
       </c>
       <c r="D24" s="19">
-        <v>942</v>
+        <v>942000</v>
       </c>
       <c r="E24" s="19">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <v>202000</v>
+      </c>
+      <c r="F24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19">
         <v>2007</v>
       </c>
       <c r="B25" s="19">
-        <v>38699</v>
+        <v>38699000</v>
       </c>
       <c r="C25" s="19">
-        <v>8582</v>
+        <v>8582000</v>
       </c>
       <c r="D25" s="19">
-        <v>2742</v>
+        <v>2742000</v>
       </c>
       <c r="E25" s="19">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>226000</v>
+      </c>
+      <c r="F25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>2008</v>
       </c>
       <c r="B26" s="19">
-        <v>60884</v>
+        <v>60884000</v>
       </c>
       <c r="C26" s="19">
-        <v>13618</v>
+        <v>13618000</v>
       </c>
       <c r="D26" s="19">
-        <v>2437</v>
+        <v>2437000</v>
       </c>
       <c r="E26" s="19">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>581000</v>
+      </c>
+      <c r="F26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="19">
         <v>2009</v>
       </c>
       <c r="B27" s="19">
-        <v>87467</v>
+        <v>87467000</v>
       </c>
       <c r="C27" s="19">
-        <v>23357</v>
+        <v>23357000</v>
       </c>
       <c r="D27" s="19">
-        <v>3707</v>
+        <v>3707000</v>
       </c>
       <c r="E27" s="19">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>503000</v>
+      </c>
+      <c r="F27"/>
+      <c r="L27"/>
+      <c r="M27"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>2010</v>
       </c>
       <c r="B28" s="19">
-        <v>7810</v>
+        <v>7810000</v>
       </c>
       <c r="C28" s="19">
-        <v>32044</v>
+        <v>32044000</v>
       </c>
       <c r="D28" s="19">
-        <v>7764</v>
+        <v>7764000</v>
       </c>
       <c r="E28" s="19">
-        <v>702</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>702000</v>
+      </c>
+      <c r="F28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="19">
         <v>2011</v>
       </c>
       <c r="B29" s="19">
-        <v>13185</v>
+        <v>13185000</v>
       </c>
       <c r="C29" s="19">
-        <v>2853</v>
+        <v>2853000</v>
       </c>
       <c r="D29" s="19">
-        <v>7258</v>
+        <v>7258000</v>
       </c>
       <c r="E29" s="19">
-        <v>1441</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1441000</v>
+      </c>
+      <c r="F29"/>
+      <c r="L29"/>
+      <c r="M29"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>2012</v>
       </c>
       <c r="B30" s="19">
-        <v>64940</v>
+        <v>64940000</v>
       </c>
       <c r="C30" s="19">
-        <v>4618</v>
+        <v>4618000</v>
       </c>
       <c r="D30" s="19">
-        <v>869</v>
+        <v>869000</v>
       </c>
       <c r="E30" s="19">
-        <v>1836</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1836000</v>
+      </c>
+      <c r="F30"/>
+      <c r="L30"/>
+      <c r="M30"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="19">
         <v>2013</v>
       </c>
       <c r="B31" s="19">
-        <v>19483</v>
+        <v>19483000</v>
       </c>
       <c r="C31" s="19">
-        <v>20991</v>
+        <v>20991000</v>
       </c>
       <c r="D31" s="19">
-        <v>1351</v>
+        <v>1351000</v>
       </c>
       <c r="E31" s="19">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>478000</v>
+      </c>
+      <c r="F31"/>
+      <c r="L31"/>
+      <c r="M31"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>2014</v>
       </c>
       <c r="B32" s="19">
-        <v>103496</v>
+        <v>103496000</v>
       </c>
       <c r="C32" s="19">
-        <v>5857</v>
+        <v>5857000</v>
       </c>
       <c r="D32" s="19">
-        <v>3580</v>
+        <v>3580000</v>
       </c>
       <c r="E32" s="19">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>264000</v>
+      </c>
+      <c r="F32"/>
+      <c r="L32"/>
+      <c r="M32"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19">
         <v>2015</v>
       </c>
       <c r="B33" s="19">
-        <v>39759</v>
+        <v>39759000</v>
       </c>
       <c r="C33" s="19">
-        <v>28070</v>
+        <v>28070000</v>
       </c>
       <c r="D33" s="19">
-        <v>1285</v>
+        <v>1285000</v>
       </c>
       <c r="E33" s="19">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>588000</v>
+      </c>
+      <c r="F33"/>
+      <c r="L33"/>
+      <c r="M33"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>2016</v>
       </c>
       <c r="B34" s="19">
-        <v>70563</v>
+        <v>70563000</v>
       </c>
       <c r="C34" s="19">
-        <v>10125</v>
+        <v>10125000</v>
       </c>
       <c r="D34" s="19">
-        <v>4592</v>
+        <v>4592000</v>
       </c>
       <c r="E34" s="19">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>261000</v>
+      </c>
+      <c r="F34"/>
+      <c r="L34"/>
+      <c r="M34"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="19">
         <v>2017</v>
       </c>
       <c r="B35" s="19">
-        <v>22784</v>
+        <v>22784000</v>
       </c>
       <c r="C35" s="19">
-        <v>17995</v>
+        <v>17995000</v>
       </c>
       <c r="D35" s="19">
-        <v>1653</v>
+        <v>1653000</v>
       </c>
       <c r="E35" s="19">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>694000</v>
+      </c>
+      <c r="F35"/>
+      <c r="L35"/>
+      <c r="M35"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>2018</v>
       </c>
       <c r="B36" s="19">
-        <v>81343</v>
+        <v>81343000</v>
       </c>
       <c r="C36" s="19">
-        <v>6022</v>
+        <v>6022000</v>
       </c>
       <c r="D36" s="19">
-        <v>2801</v>
+        <v>2801000</v>
       </c>
       <c r="E36" s="19">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>315000</v>
+      </c>
+      <c r="F36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="19">
         <v>2019</v>
       </c>
       <c r="B37" s="19">
-        <v>107180</v>
+        <v>107180000</v>
       </c>
       <c r="C37" s="19">
-        <v>23717</v>
+        <v>23717000</v>
       </c>
       <c r="D37" s="19">
-        <v>1356</v>
+        <v>1356000</v>
       </c>
       <c r="E37" s="19">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+        <v>399000</v>
+      </c>
+      <c r="F37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>2020</v>
       </c>
       <c r="B38" s="19">
-        <v>63647</v>
+        <v>63647000</v>
       </c>
       <c r="C38" s="19">
-        <v>32394</v>
+        <v>32394000</v>
       </c>
       <c r="D38" s="19">
-        <v>4839</v>
+        <v>4839000</v>
       </c>
       <c r="E38" s="19">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>272000</v>
+      </c>
+      <c r="F38"/>
+      <c r="L38"/>
+      <c r="M38"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="19">
         <v>2021</v>
       </c>
       <c r="B39" s="19">
-        <v>25638</v>
+        <v>25638000</v>
       </c>
       <c r="C39" s="19">
-        <v>16952</v>
+        <v>16952000</v>
       </c>
       <c r="D39" s="19">
-        <v>5511</v>
+        <v>5511000</v>
       </c>
       <c r="E39" s="19">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>775000</v>
+      </c>
+      <c r="F39"/>
+      <c r="L39"/>
+      <c r="M39"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>2022</v>
       </c>
       <c r="B40" s="19">
-        <v>48250</v>
+        <v>48250000</v>
       </c>
       <c r="C40" s="19">
-        <v>8107</v>
+        <v>8107000</v>
       </c>
       <c r="D40" s="19">
-        <v>2731</v>
+        <v>2731000</v>
       </c>
       <c r="E40" s="19">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>872000</v>
+      </c>
+      <c r="F40"/>
+      <c r="L40"/>
+      <c r="M40"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="19">
         <v>2023</v>
       </c>
       <c r="B41" s="19">
-        <v>9453</v>
+        <v>9453000</v>
       </c>
       <c r="C41" s="19">
-        <v>13367</v>
+        <v>13367000</v>
       </c>
       <c r="D41" s="19">
-        <v>1603</v>
+        <v>1603000</v>
       </c>
       <c r="E41" s="19">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+        <v>489000</v>
+      </c>
+      <c r="F41"/>
+      <c r="L41"/>
+      <c r="M41"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>2024</v>
       </c>
       <c r="B42" s="19">
-        <v>8851</v>
+        <v>8851000</v>
       </c>
       <c r="C42" s="19">
-        <v>2043</v>
+        <v>2043000</v>
       </c>
       <c r="D42" s="19">
-        <v>2331</v>
+        <v>2331000</v>
       </c>
       <c r="E42" s="19">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+        <v>343000</v>
+      </c>
+      <c r="F42"/>
+      <c r="L42"/>
+      <c r="M42"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="19">
         <v>2025</v>
       </c>
       <c r="B43" s="19">
-        <v>10312</v>
+        <v>10312000</v>
       </c>
       <c r="C43" s="19">
-        <v>2576</v>
+        <v>2576000</v>
       </c>
       <c r="D43" s="19">
-        <v>486</v>
+        <v>486000</v>
       </c>
       <c r="E43" s="19">
-        <v>445</v>
-      </c>
+        <v>445000</v>
+      </c>
+      <c r="F43"/>
+      <c r="L43"/>
+      <c r="M43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>